<commit_message>
add fitur cek status
</commit_message>
<xml_diff>
--- a/public/template/template_bulk_agi.xlsx
+++ b/public/template/template_bulk_agi.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Pemograman\laragon\www\apuppt\public\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\Pemograman\laragon\www\cekstatus\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FFB7A3-310D-4C48-AC6B-8D0DE1437831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57113671-410E-4AC7-A7E7-D3ED113EF726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -409,7 +409,7 @@
     <col min="4" max="4" width="10.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -432,10 +432,10 @@
       <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="I1" s="1" t="s">

</xml_diff>